<commit_message>
Cliente feedback batch 1: white cast → efecto mimo, SPF → FPS (total), lado a lado → frente a frente, sin/con compromiso, FAQ devoluciones (no abiertos), nota INCI, descripción en comparador, ortografía nosotros, Excel tags actualizado
</commit_message>
<xml_diff>
--- a/Quiz-Sistema-de-Tags.xlsx
+++ b/Quiz-Sistema-de-Tags.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Productos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lógica del Quiz" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cómo usar este Excel" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lógica del Quiz" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cómo usar este Excel" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -866,7 +866,7 @@
       </c>
       <c r="Y5" s="11" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z5" s="10" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="Y6" s="15" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z6" s="14" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="Y7" s="11" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z7" s="10" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="Y8" s="15" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z8" s="14" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="Y9" s="11" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z9" s="10" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="Y10" s="15" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z10" s="14" t="inlineStr">
@@ -1462,7 +1462,7 @@
       <c r="X11" s="11" t="inlineStr"/>
       <c r="Y11" s="11" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z11" s="10" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="Y12" s="15" t="inlineStr">
         <is>
-          <t>SPF</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="Z12" s="14" t="inlineStr">
@@ -2599,7 +2599,7 @@
       <c r="A18" s="11" t="inlineStr"/>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Maquillaje + SPF acabado mate</t>
+          <t>Maquillaje + FPS acabado mate</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Solo aplica a SPFs con compatibilidad maquillaje</t>
+          <t>Solo aplica a FPSs con compatibilidad maquillaje</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       <c r="A20" s="11" t="inlineStr"/>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>No usa SPF + producto es SPF</t>
+          <t>No usa FPS + producto es FPS</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
@@ -2743,7 +2743,7 @@
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>El quiz arma una rutina de 4 productos: 1 Limpiador + 1 Suero + 1 Crema + 1 SPF.</t>
+          <t>El quiz arma una rutina de 4 productos: 1 Limpiador + 1 Suero + 1 Crema + 1 FPS.</t>
         </is>
       </c>
     </row>

</xml_diff>